<commit_message>
fix(scripts): distinct words for the length and width columns
The column lookup is case-insensitive, so headers of „L REAL" and „l REAL"
resolved to the same column and every width came back equal to its length —
PAT-PAUL-2000X1600 read as 2000×2000. Romanian keeps L and l apart as
different quantities; a case-folding string match does not.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dimensiuni-reale.xlsx
+++ b/docs/dimensiuni-reale.xlsx
@@ -25,25 +25,25 @@
     <t>Dimensiune</t>
   </si>
   <si>
-    <t>L acum</t>
-  </si>
-  <si>
-    <t>l acum</t>
-  </si>
-  <si>
-    <t>H acum</t>
+    <t>Lungime acum</t>
+  </si>
+  <si>
+    <t>Latime acum</t>
+  </si>
+  <si>
+    <t>Inaltime acum</t>
   </si>
   <si>
     <t>Din import?</t>
   </si>
   <si>
-    <t>L REAL  ←</t>
-  </si>
-  <si>
-    <t>l REAL  ←</t>
-  </si>
-  <si>
-    <t>H REAL  ←</t>
+    <t>Lungime REALA  ←</t>
+  </si>
+  <si>
+    <t>Latime REALA  ←</t>
+  </si>
+  <si>
+    <t>Inaltime REALA  ←</t>
   </si>
   <si>
     <t>Produs finit în SAGA</t>

</xml_diff>